<commit_message>
fix lỗi tự submit form khi tìm sản phẩm
</commit_message>
<xml_diff>
--- a/public/files/template/Nhap_phu_phi_don_hang.xlsx
+++ b/public/files/template/Nhap_phu_phi_don_hang.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC54052-C04A-4BFE-97D5-5F3E21146663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DC344A-0EEE-47EB-8B75-FAE2E1643E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28095" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,6 @@
     <t>Phụ phí</t>
   </si>
   <si>
-    <t>Ngày thanh toán</t>
-  </si>
-  <si>
     <t>12/04/2024</t>
   </si>
   <si>
@@ -65,6 +62,9 @@
   </si>
   <si>
     <t>S14206351.MB9-12-F0.1934603753</t>
+  </si>
+  <si>
+    <t>Ngày xuất hàng</t>
   </si>
 </sst>
 </file>
@@ -501,7 +501,7 @@
         <v>8</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -509,7 +509,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>3</v>
@@ -518,7 +518,7 @@
         <v>280000</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -526,7 +526,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>4</v>
@@ -535,7 +535,7 @@
         <v>280000</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -543,7 +543,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -552,7 +552,7 @@
         <v>280000</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -560,7 +560,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
@@ -569,7 +569,7 @@
         <v>170000</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -577,7 +577,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>7</v>
@@ -586,7 +586,7 @@
         <v>180000</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>